<commit_message>
Add Mapper and Scheduler to software page and CV
Added both to the javascript section of software.xlsx and to the
Software (selected) section of JRM_CV.tex.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/software.xlsx
+++ b/data/software.xlsx
@@ -672,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -699,6 +699,11 @@
           <t>github_link</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>docs_link</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="51" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -714,6 +719,50 @@
       <c r="C2" s="9" t="inlineStr">
         <is>
           <t>https://github.com/ContextLab/autoFR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mapper</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Map out an approximation of everything you know by answering multiple-choice quiz questions.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/mapper</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://context-lab.com/mapper/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Scheduler</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A self-hosted appointment scheduling system like YouCanBook.me or Calendly, but free, open-source, and fully under your control.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://github.com/ContextLab/scheduler</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://cdl-scheduler.readthedocs.io/</t>
         </is>
       </c>
     </row>

</xml_diff>